<commit_message>
Updated liga mx results tab
</commit_message>
<xml_diff>
--- a/LigaMX/predictions/model_compareLMX.xlsx
+++ b/LigaMX/predictions/model_compareLMX.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\LigaMX\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61060F73-0BFA-4077-857E-2071008BE5C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FBA626-CB34-4599-A0F5-088D2F4312AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-78" yWindow="0" windowWidth="11676" windowHeight="12318" activeTab="1" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Models" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="87">
   <si>
     <t>Model</t>
   </si>
@@ -244,6 +244,60 @@
   </si>
   <si>
     <t>cat_lgbm_xgb</t>
+  </si>
+  <si>
+    <t>Puebla Loss</t>
+  </si>
+  <si>
+    <t>Tijuana Loss</t>
+  </si>
+  <si>
+    <t>Atlas Win</t>
+  </si>
+  <si>
+    <t>Puebla Win</t>
+  </si>
+  <si>
+    <t>Pachuca Win</t>
+  </si>
+  <si>
+    <t>FC Juarez Loss</t>
+  </si>
+  <si>
+    <t>America Loss</t>
+  </si>
+  <si>
+    <t>Tigres UANL Win</t>
+  </si>
+  <si>
+    <t>Tigres UANL Loss</t>
+  </si>
+  <si>
+    <t>Toluca Win</t>
+  </si>
+  <si>
+    <t>Necaxa Win</t>
+  </si>
+  <si>
+    <t>Pacucha Win</t>
+  </si>
+  <si>
+    <t>Queretaro Win</t>
+  </si>
+  <si>
+    <t>Toluca Loss</t>
+  </si>
+  <si>
+    <t>FC Juarez Win</t>
+  </si>
+  <si>
+    <t>Pachuca Loss</t>
+  </si>
+  <si>
+    <t>Santos Laguna Win</t>
+  </si>
+  <si>
+    <t>Cuartos</t>
   </si>
 </sst>
 </file>
@@ -432,7 +486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -470,7 +524,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1122,7 +1175,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="1">
@@ -1570,7 +1623,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2AB4D39-76AB-4A8D-8A49-E2E912416120}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E162"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="2" max="3" width="13.578125" bestFit="1" customWidth="1"/>
@@ -1596,50 +1649,50 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A2">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
         <v>47</v>
@@ -1647,67 +1700,67 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
         <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="E8" t="s">
         <v>45</v>
@@ -1715,288 +1768,1708 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
         <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E11" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="E12" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
         <v>35</v>
       </c>
-      <c r="C13" t="s">
-        <v>27</v>
-      </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E13" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="E15" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="D16" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="E16" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="D17" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E17" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>76</v>
       </c>
       <c r="E18" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D19" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E19" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>53</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>25</v>
+        <v>38</v>
+      </c>
+      <c r="D21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>26</v>
+        <v>35</v>
+      </c>
+      <c r="D22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A23">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C23" t="s">
         <v>43</v>
       </c>
+      <c r="D23" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A24">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
+        <v>54</v>
+      </c>
+      <c r="E24" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A25">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>50</v>
+      </c>
+      <c r="D25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A26">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="C26" t="s">
-        <v>53</v>
+        <v>24</v>
+      </c>
+      <c r="D26" t="s">
+        <v>66</v>
+      </c>
+      <c r="E26" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A27">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>35</v>
+        <v>27</v>
+      </c>
+      <c r="D27" t="s">
+        <v>34</v>
+      </c>
+      <c r="E27" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A28">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" t="s">
+        <v>75</v>
+      </c>
+      <c r="E29" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" t="s">
+        <v>39</v>
+      </c>
+      <c r="D30" t="s">
+        <v>63</v>
+      </c>
+      <c r="E30" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" t="s">
+        <v>71</v>
+      </c>
+      <c r="E31" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" t="s">
+        <v>50</v>
+      </c>
+      <c r="D32" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" t="s">
+        <v>32</v>
+      </c>
+      <c r="D33" t="s">
+        <v>74</v>
+      </c>
+      <c r="E33" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" t="s">
+        <v>58</v>
+      </c>
+      <c r="E34" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35">
+        <v>4</v>
+      </c>
+      <c r="B35" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" t="s">
+        <v>59</v>
+      </c>
+      <c r="E35" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36">
+        <v>4</v>
+      </c>
+      <c r="B36" t="s">
+        <v>35</v>
+      </c>
+      <c r="C36" t="s">
+        <v>33</v>
+      </c>
+      <c r="D36" t="s">
+        <v>37</v>
+      </c>
+      <c r="E36" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37">
+        <v>4</v>
+      </c>
+      <c r="B37" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" t="s">
+        <v>30</v>
+      </c>
+      <c r="D37" t="s">
+        <v>45</v>
+      </c>
+      <c r="E37" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A38">
+        <v>5</v>
+      </c>
+      <c r="B38" t="s">
+        <v>38</v>
+      </c>
+      <c r="C38" t="s">
+        <v>43</v>
+      </c>
+      <c r="D38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E38" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A39">
+        <v>5</v>
+      </c>
+      <c r="B39" t="s">
+        <v>50</v>
+      </c>
+      <c r="C39" t="s">
+        <v>32</v>
+      </c>
+      <c r="D39" t="s">
+        <v>82</v>
+      </c>
+      <c r="E39" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A40">
+        <v>5</v>
+      </c>
+      <c r="B40" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" t="s">
+        <v>52</v>
+      </c>
+      <c r="D40" t="s">
+        <v>76</v>
+      </c>
+      <c r="E40" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A41">
+        <v>5</v>
+      </c>
+      <c r="B41" t="s">
+        <v>29</v>
+      </c>
+      <c r="C41" t="s">
+        <v>24</v>
+      </c>
+      <c r="D41" t="s">
+        <v>79</v>
+      </c>
+      <c r="E41" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A42">
+        <v>5</v>
+      </c>
+      <c r="B42" t="s">
+        <v>33</v>
+      </c>
+      <c r="C42" t="s">
+        <v>27</v>
+      </c>
+      <c r="D42" t="s">
+        <v>66</v>
+      </c>
+      <c r="E42" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A43">
+        <v>5</v>
+      </c>
+      <c r="B43" t="s">
+        <v>26</v>
+      </c>
+      <c r="C43" t="s">
+        <v>39</v>
+      </c>
+      <c r="D43" t="s">
+        <v>65</v>
+      </c>
+      <c r="E43" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A44">
+        <v>5</v>
+      </c>
+      <c r="B44" t="s">
+        <v>53</v>
+      </c>
+      <c r="C44" t="s">
+        <v>25</v>
+      </c>
+      <c r="D44" t="s">
+        <v>62</v>
+      </c>
+      <c r="E44" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A45">
+        <v>5</v>
+      </c>
+      <c r="B45" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" t="s">
+        <v>80</v>
+      </c>
+      <c r="E45" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A46">
+        <v>5</v>
+      </c>
+      <c r="B46" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" t="s">
+        <v>35</v>
+      </c>
+      <c r="D46" t="s">
+        <v>51</v>
+      </c>
+      <c r="E46" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A47">
+        <v>6</v>
+      </c>
+      <c r="B47" t="s">
+        <v>36</v>
+      </c>
+      <c r="C47" t="s">
+        <v>53</v>
+      </c>
+      <c r="D47" t="s">
+        <v>80</v>
+      </c>
+      <c r="E47" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A48">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
+        <v>24</v>
+      </c>
+      <c r="C48" t="s">
+        <v>38</v>
+      </c>
+      <c r="D48" t="s">
+        <v>63</v>
+      </c>
+      <c r="E48" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A49">
+        <v>6</v>
+      </c>
+      <c r="B49" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" t="s">
+        <v>25</v>
+      </c>
+      <c r="D49" t="s">
+        <v>69</v>
+      </c>
+      <c r="E49" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A50">
+        <v>6</v>
+      </c>
+      <c r="B50" t="s">
+        <v>50</v>
+      </c>
+      <c r="C50" t="s">
+        <v>33</v>
+      </c>
+      <c r="D50" t="s">
+        <v>78</v>
+      </c>
+      <c r="E50" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A51">
+        <v>6</v>
+      </c>
+      <c r="B51" t="s">
+        <v>32</v>
+      </c>
+      <c r="C51" t="s">
+        <v>30</v>
+      </c>
+      <c r="D51" t="s">
+        <v>34</v>
+      </c>
+      <c r="E51" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A52">
+        <v>6</v>
+      </c>
+      <c r="B52" t="s">
+        <v>52</v>
+      </c>
+      <c r="C52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52" t="s">
+        <v>54</v>
+      </c>
+      <c r="E52" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A53">
+        <v>6</v>
+      </c>
+      <c r="B53" t="s">
+        <v>44</v>
+      </c>
+      <c r="C53" t="s">
+        <v>29</v>
+      </c>
+      <c r="D53" t="s">
+        <v>74</v>
+      </c>
+      <c r="E53" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54">
+        <v>6</v>
+      </c>
+      <c r="B54" t="s">
+        <v>35</v>
+      </c>
+      <c r="C54" t="s">
+        <v>43</v>
+      </c>
+      <c r="D54" t="s">
+        <v>37</v>
+      </c>
+      <c r="E54" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A55">
+        <v>6</v>
+      </c>
+      <c r="B55" t="s">
+        <v>39</v>
+      </c>
+      <c r="C55" t="s">
+        <v>49</v>
+      </c>
+      <c r="D55" t="s">
+        <v>40</v>
+      </c>
+      <c r="E55" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A56">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A57">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A58">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A59">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A60">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A61">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A62">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A63">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A64">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A65">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A66">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A67">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A68">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A69">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A70">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A71">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A72">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A73">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A74">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A75">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A76">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A77">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A78">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A79">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A80">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A81">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A82">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A83">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A84">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A85">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A86">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A87">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A88">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A89">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A90">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A91">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A92">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A93">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A94">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A95">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A96">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A97">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A98">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A99">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A100">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A101">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A102">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A103">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A104">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A105">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A106">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A107">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A108">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A109">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A110">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A111">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A112">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A113">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A114">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A115">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A116">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A117">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A118">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A119">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A120">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A121">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A122">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A123">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A124">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A125">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A126">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A127">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A128">
+        <v>15</v>
+      </c>
+      <c r="B128" t="s">
+        <v>24</v>
+      </c>
+      <c r="C128" t="s">
+        <v>25</v>
+      </c>
+      <c r="D128" t="s">
+        <v>64</v>
+      </c>
+      <c r="E128" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A129">
+        <v>15</v>
+      </c>
+      <c r="B129" t="s">
+        <v>26</v>
+      </c>
+      <c r="C129" t="s">
+        <v>38</v>
+      </c>
+      <c r="D129" t="s">
+        <v>28</v>
+      </c>
+      <c r="E129" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A130">
+        <v>15</v>
+      </c>
+      <c r="B130" t="s">
+        <v>29</v>
+      </c>
+      <c r="C130" t="s">
+        <v>30</v>
+      </c>
+      <c r="D130" t="s">
+        <v>31</v>
+      </c>
+      <c r="E130" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A131">
+        <v>15</v>
+      </c>
+      <c r="B131" t="s">
+        <v>32</v>
+      </c>
+      <c r="C131" t="s">
+        <v>33</v>
+      </c>
+      <c r="D131" t="s">
+        <v>34</v>
+      </c>
+      <c r="E131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A132">
+        <v>15</v>
+      </c>
+      <c r="B132" t="s">
+        <v>35</v>
+      </c>
+      <c r="C132" t="s">
+        <v>36</v>
+      </c>
+      <c r="D132" t="s">
+        <v>37</v>
+      </c>
+      <c r="E132" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A133">
+        <v>15</v>
+      </c>
+      <c r="B133" t="s">
+        <v>39</v>
+      </c>
+      <c r="C133" t="s">
+        <v>27</v>
+      </c>
+      <c r="D133" t="s">
+        <v>40</v>
+      </c>
+      <c r="E133" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A134">
+        <v>15</v>
+      </c>
+      <c r="B134" t="s">
+        <v>43</v>
+      </c>
+      <c r="C134" t="s">
+        <v>44</v>
+      </c>
+      <c r="D134" t="s">
+        <v>45</v>
+      </c>
+      <c r="E134" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A135">
+        <v>15</v>
+      </c>
+      <c r="B135" t="s">
+        <v>49</v>
+      </c>
+      <c r="C135" t="s">
+        <v>50</v>
+      </c>
+      <c r="D135" t="s">
+        <v>47</v>
+      </c>
+      <c r="E135" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A136">
+        <v>15</v>
+      </c>
+      <c r="B136" t="s">
+        <v>52</v>
+      </c>
+      <c r="C136" t="s">
+        <v>53</v>
+      </c>
+      <c r="D136" t="s">
+        <v>54</v>
+      </c>
+      <c r="E136" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A137">
+        <v>16</v>
+      </c>
+      <c r="B137" t="s">
+        <v>25</v>
+      </c>
+      <c r="C137" t="s">
+        <v>44</v>
+      </c>
+      <c r="D137" t="s">
+        <v>58</v>
+      </c>
+      <c r="E137" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A138">
+        <v>16</v>
+      </c>
+      <c r="B138" t="s">
+        <v>38</v>
+      </c>
+      <c r="C138" t="s">
+        <v>32</v>
+      </c>
+      <c r="D138" t="s">
+        <v>59</v>
+      </c>
+      <c r="E138" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A139">
+        <v>16</v>
+      </c>
+      <c r="B139" t="s">
+        <v>35</v>
+      </c>
+      <c r="C139" t="s">
+        <v>27</v>
+      </c>
+      <c r="D139" t="s">
+        <v>37</v>
+      </c>
+      <c r="E139" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A140">
+        <v>16</v>
+      </c>
+      <c r="B140" t="s">
+        <v>60</v>
+      </c>
+      <c r="C140" t="s">
+        <v>49</v>
+      </c>
+      <c r="D140" t="s">
+        <v>45</v>
+      </c>
+      <c r="E140" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A141">
+        <v>16</v>
+      </c>
+      <c r="B141" t="s">
+        <v>53</v>
+      </c>
+      <c r="C141" t="s">
+        <v>30</v>
+      </c>
+      <c r="D141" t="s">
+        <v>62</v>
+      </c>
+      <c r="E141" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A142">
+        <v>16</v>
+      </c>
+      <c r="B142" t="s">
+        <v>24</v>
+      </c>
+      <c r="C142" t="s">
+        <v>52</v>
+      </c>
+      <c r="D142" t="s">
+        <v>63</v>
+      </c>
+      <c r="E142" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A143">
+        <v>16</v>
+      </c>
+      <c r="B143" t="s">
+        <v>26</v>
+      </c>
+      <c r="C143" t="s">
+        <v>50</v>
+      </c>
+      <c r="D143" t="s">
+        <v>65</v>
+      </c>
+      <c r="E143" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A144">
+        <v>16</v>
+      </c>
+      <c r="B144" t="s">
+        <v>29</v>
+      </c>
+      <c r="C144" t="s">
+        <v>39</v>
+      </c>
+      <c r="D144" t="s">
+        <v>31</v>
+      </c>
+      <c r="E144" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A145">
+        <v>16</v>
+      </c>
+      <c r="B145" t="s">
+        <v>33</v>
+      </c>
+      <c r="C145" t="s">
+        <v>36</v>
+      </c>
+      <c r="D145" t="s">
+        <v>66</v>
+      </c>
+      <c r="E145" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A146">
         <v>17</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B146" t="s">
+        <v>27</v>
+      </c>
+      <c r="C146" t="s">
+        <v>38</v>
+      </c>
+      <c r="D146" t="s">
+        <v>69</v>
+      </c>
+      <c r="E146" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A147">
+        <v>17</v>
+      </c>
+      <c r="B147" t="s">
+        <v>36</v>
+      </c>
+      <c r="C147" t="s">
+        <v>25</v>
+      </c>
+      <c r="D147" t="s">
+        <v>47</v>
+      </c>
+      <c r="E147" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A148">
+        <v>17</v>
+      </c>
+      <c r="B148" t="s">
+        <v>30</v>
+      </c>
+      <c r="C148" t="s">
+        <v>26</v>
+      </c>
+      <c r="D148" t="s">
+        <v>76</v>
+      </c>
+      <c r="E148" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A149">
+        <v>17</v>
+      </c>
+      <c r="B149" t="s">
+        <v>50</v>
+      </c>
+      <c r="C149" t="s">
+        <v>43</v>
+      </c>
+      <c r="D149" t="s">
+        <v>47</v>
+      </c>
+      <c r="E149" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A150">
+        <v>17</v>
+      </c>
+      <c r="B150" t="s">
+        <v>39</v>
+      </c>
+      <c r="C150" t="s">
+        <v>33</v>
+      </c>
+      <c r="D150" t="s">
+        <v>40</v>
+      </c>
+      <c r="E150" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A151">
+        <v>17</v>
+      </c>
+      <c r="B151" t="s">
+        <v>44</v>
+      </c>
+      <c r="C151" t="s">
+        <v>24</v>
+      </c>
+      <c r="D151" t="s">
+        <v>83</v>
+      </c>
+      <c r="E151" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A152">
+        <v>17</v>
+      </c>
+      <c r="B152" t="s">
+        <v>49</v>
+      </c>
+      <c r="C152" t="s">
+        <v>53</v>
+      </c>
+      <c r="D152" t="s">
+        <v>51</v>
+      </c>
+      <c r="E152" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A153">
+        <v>17</v>
+      </c>
+      <c r="B153" t="s">
+        <v>52</v>
+      </c>
+      <c r="C153" t="s">
+        <v>35</v>
+      </c>
+      <c r="D153" t="s">
+        <v>54</v>
+      </c>
+      <c r="E153" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A154">
+        <v>17</v>
+      </c>
+      <c r="B154" t="s">
         <v>32</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C154" t="s">
         <v>29</v>
+      </c>
+      <c r="D154" t="s">
+        <v>34</v>
+      </c>
+      <c r="E154" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A155" t="s">
+        <v>86</v>
+      </c>
+      <c r="B155" t="s">
+        <v>30</v>
+      </c>
+      <c r="C155" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A156" t="s">
+        <v>86</v>
+      </c>
+      <c r="B156" t="s">
+        <v>53</v>
+      </c>
+      <c r="C156" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A157" t="s">
+        <v>86</v>
+      </c>
+      <c r="B157" t="s">
+        <v>49</v>
+      </c>
+      <c r="C157" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A158" t="s">
+        <v>86</v>
+      </c>
+      <c r="B158" t="s">
+        <v>50</v>
+      </c>
+      <c r="C158" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A159" t="s">
+        <v>86</v>
+      </c>
+      <c r="B159" t="s">
+        <v>39</v>
+      </c>
+      <c r="C159" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A160" t="s">
+        <v>86</v>
+      </c>
+      <c r="B160" t="s">
+        <v>32</v>
+      </c>
+      <c r="C160" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A161" t="s">
+        <v>86</v>
+      </c>
+      <c r="B161" t="s">
+        <v>36</v>
+      </c>
+      <c r="C161" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A162" t="s">
+        <v>86</v>
+      </c>
+      <c r="B162" t="s">
+        <v>25</v>
+      </c>
+      <c r="C162" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Results page for Liga MX
</commit_message>
<xml_diff>
--- a/LigaMX/predictions/model_compareLMX.xlsx
+++ b/LigaMX/predictions/model_compareLMX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\LigaMX\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A02D5F-2B39-4E95-A814-074993E68206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72638C44-8595-4505-BEB3-D2CF2ED50218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="90">
   <si>
     <t>Model</t>
   </si>
@@ -3533,20 +3533,68 @@
       <c r="A163" t="s">
         <v>88</v>
       </c>
+      <c r="B163" t="s">
+        <v>32</v>
+      </c>
+      <c r="C163" t="s">
+        <v>39</v>
+      </c>
+      <c r="D163" t="s">
+        <v>47</v>
+      </c>
+      <c r="E163" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A164" t="s">
         <v>88</v>
       </c>
+      <c r="B164" t="s">
+        <v>36</v>
+      </c>
+      <c r="C164" t="s">
+        <v>25</v>
+      </c>
+      <c r="D164" t="s">
+        <v>80</v>
+      </c>
+      <c r="E164" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A165" t="s">
         <v>88</v>
       </c>
+      <c r="B165" t="s">
+        <v>39</v>
+      </c>
+      <c r="C165" t="s">
+        <v>32</v>
+      </c>
+      <c r="D165" t="s">
+        <v>47</v>
+      </c>
+      <c r="E165" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A166" t="s">
         <v>88</v>
+      </c>
+      <c r="B166" t="s">
+        <v>25</v>
+      </c>
+      <c r="C166" t="s">
+        <v>36</v>
+      </c>
+      <c r="D166" t="s">
+        <v>58</v>
+      </c>
+      <c r="E166" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.55000000000000004">

</xml_diff>